<commit_message>
Fiks sensitivitetsanalyse og småfeil i analysescript og rapport
- Sensitivitet: rekn frekvensavvik på nytt per (S, h)-kombinasjon i staden for å bruke base-case FREQ_AVVIK_PCT
- Sensitivitet: bruk ΔTC×g-modell (konsistent med modul 7) i staden for gammal f×S×r-formel
- Versjonsnummer i print: v2.5 → v2.7
- Kommentarreferanse: D-03 → D-06 (MSEG_STATUS)
- Rapport: rett parameterliste i sensitivitetsomtale frå «S, h og g» til «S, h og τ_f»
- Bygg Word-dokument på nytt

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/006 Analyse/LOG650_Resultater.xlsx
+++ b/006 Analyse/LOG650_Resultater.xlsx
@@ -4952,13 +4952,13 @@
     <t>ΔTC total (kr/år)</t>
   </si>
   <si>
-    <t>B_total base (kr/år)</t>
+    <t>B_HVFS base g=75% (kr/år)</t>
   </si>
   <si>
     <t>Sensitivitetsanalyse – 27 scenariokombiner (S × h × τ_f)</t>
   </si>
   <si>
-    <t>S ∈ {500, 750, 1000} kr  |  h ∈ {0,15, 0,20, 0,25}  |  τ_f ∈ {1,25, 1,50, 2,00}  |  r = 12% (base case)</t>
+    <t>S ∈ {500, 750, 1000} kr  |  h ∈ {0,15, 0,20, 0,25}  |  τ_f ∈ {1,25, 1,50, 2,00}  |  g = 75% (base case)</t>
   </si>
 </sst>
 </file>
@@ -56355,19 +56355,19 @@
         <v>1.25</v>
       </c>
       <c r="D5">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="E5">
         <v>54</v>
       </c>
       <c r="F5">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="G5">
         <v>1602464</v>
       </c>
       <c r="H5">
-        <v>105060</v>
+        <v>284941</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -56381,19 +56381,19 @@
         <v>1.5</v>
       </c>
       <c r="D6">
-        <v>356</v>
+        <v>350</v>
       </c>
       <c r="E6">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="F6">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G6">
         <v>1602464</v>
       </c>
       <c r="H6">
-        <v>105060</v>
+        <v>284305</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -56407,10 +56407,10 @@
         <v>2</v>
       </c>
       <c r="D7">
-        <v>306</v>
+        <v>294</v>
       </c>
       <c r="E7">
-        <v>181</v>
+        <v>193</v>
       </c>
       <c r="F7">
         <v>0</v>
@@ -56419,7 +56419,7 @@
         <v>1602464</v>
       </c>
       <c r="H7">
-        <v>105060</v>
+        <v>263896</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -56433,19 +56433,19 @@
         <v>1.25</v>
       </c>
       <c r="D8">
-        <v>379</v>
+        <v>353</v>
       </c>
       <c r="E8">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="F8">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="G8">
         <v>1770359</v>
       </c>
       <c r="H8">
-        <v>105060</v>
+        <v>244538</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -56459,19 +56459,19 @@
         <v>1.5</v>
       </c>
       <c r="D9">
-        <v>356</v>
+        <v>326</v>
       </c>
       <c r="E9">
-        <v>100</v>
+        <v>122</v>
       </c>
       <c r="F9">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="G9">
         <v>1770359</v>
       </c>
       <c r="H9">
-        <v>105060</v>
+        <v>241543</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -56485,10 +56485,10 @@
         <v>2</v>
       </c>
       <c r="D10">
-        <v>306</v>
+        <v>269</v>
       </c>
       <c r="E10">
-        <v>181</v>
+        <v>218</v>
       </c>
       <c r="F10">
         <v>0</v>
@@ -56497,7 +56497,7 @@
         <v>1770359</v>
       </c>
       <c r="H10">
-        <v>105060</v>
+        <v>218615</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -56511,19 +56511,19 @@
         <v>1.25</v>
       </c>
       <c r="D11">
-        <v>379</v>
+        <v>337</v>
       </c>
       <c r="E11">
-        <v>54</v>
+        <v>71</v>
       </c>
       <c r="F11">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="G11">
         <v>1968108</v>
       </c>
       <c r="H11">
-        <v>105060</v>
+        <v>211826</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -56537,19 +56537,19 @@
         <v>1.5</v>
       </c>
       <c r="D12">
-        <v>356</v>
+        <v>302</v>
       </c>
       <c r="E12">
-        <v>100</v>
+        <v>142</v>
       </c>
       <c r="F12">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="G12">
         <v>1968108</v>
       </c>
       <c r="H12">
-        <v>105060</v>
+        <v>206617</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -56563,10 +56563,10 @@
         <v>2</v>
       </c>
       <c r="D13">
-        <v>306</v>
+        <v>232</v>
       </c>
       <c r="E13">
-        <v>181</v>
+        <v>255</v>
       </c>
       <c r="F13">
         <v>0</v>
@@ -56575,7 +56575,7 @@
         <v>1968108</v>
       </c>
       <c r="H13">
-        <v>105060</v>
+        <v>176374</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -56589,19 +56589,19 @@
         <v>1.25</v>
       </c>
       <c r="D14">
-        <v>379</v>
+        <v>400</v>
       </c>
       <c r="E14">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="F14">
-        <v>54</v>
+        <v>41</v>
       </c>
       <c r="G14">
         <v>2221932</v>
       </c>
       <c r="H14">
-        <v>157590</v>
+        <v>508107</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -56615,19 +56615,19 @@
         <v>1.5</v>
       </c>
       <c r="D15">
-        <v>356</v>
+        <v>377</v>
       </c>
       <c r="E15">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="F15">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G15">
         <v>2221932</v>
       </c>
       <c r="H15">
-        <v>157590</v>
+        <v>508107</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -56641,10 +56641,10 @@
         <v>2</v>
       </c>
       <c r="D16">
-        <v>306</v>
+        <v>332</v>
       </c>
       <c r="E16">
-        <v>181</v>
+        <v>155</v>
       </c>
       <c r="F16">
         <v>0</v>
@@ -56653,7 +56653,7 @@
         <v>2221932</v>
       </c>
       <c r="H16">
-        <v>157590</v>
+        <v>493952</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -56679,7 +56679,7 @@
         <v>2333433</v>
       </c>
       <c r="H17">
-        <v>157590</v>
+        <v>451519</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -56705,7 +56705,7 @@
         <v>2333433</v>
       </c>
       <c r="H18">
-        <v>157590</v>
+        <v>451519</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -56731,7 +56731,7 @@
         <v>2333433</v>
       </c>
       <c r="H19">
-        <v>157590</v>
+        <v>425702</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -56745,19 +56745,19 @@
         <v>1.25</v>
       </c>
       <c r="D20">
-        <v>379</v>
+        <v>366</v>
       </c>
       <c r="E20">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="F20">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="G20">
         <v>2481499</v>
       </c>
       <c r="H20">
-        <v>157590</v>
+        <v>405479</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -56771,19 +56771,19 @@
         <v>1.5</v>
       </c>
       <c r="D21">
-        <v>356</v>
+        <v>340</v>
       </c>
       <c r="E21">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="F21">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="G21">
         <v>2481499</v>
       </c>
       <c r="H21">
-        <v>157590</v>
+        <v>400268</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -56797,10 +56797,10 @@
         <v>2</v>
       </c>
       <c r="D22">
-        <v>306</v>
+        <v>282</v>
       </c>
       <c r="E22">
-        <v>181</v>
+        <v>205</v>
       </c>
       <c r="F22">
         <v>0</v>
@@ -56809,7 +56809,7 @@
         <v>2481499</v>
       </c>
       <c r="H22">
-        <v>157590</v>
+        <v>367520</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -56823,19 +56823,19 @@
         <v>1.25</v>
       </c>
       <c r="D23">
-        <v>379</v>
+        <v>422</v>
       </c>
       <c r="E23">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="F23">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="G23">
         <v>2898617</v>
       </c>
       <c r="H23">
-        <v>210120</v>
+        <v>747776</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -56849,19 +56849,19 @@
         <v>1.5</v>
       </c>
       <c r="D24">
-        <v>356</v>
+        <v>397</v>
       </c>
       <c r="E24">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="F24">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="G24">
         <v>2898617</v>
       </c>
       <c r="H24">
-        <v>210120</v>
+        <v>747776</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -56875,10 +56875,10 @@
         <v>2</v>
       </c>
       <c r="D25">
-        <v>306</v>
+        <v>356</v>
       </c>
       <c r="E25">
-        <v>181</v>
+        <v>131</v>
       </c>
       <c r="F25">
         <v>0</v>
@@ -56887,7 +56887,7 @@
         <v>2898617</v>
       </c>
       <c r="H25">
-        <v>210120</v>
+        <v>747776</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -56901,19 +56901,19 @@
         <v>1.25</v>
       </c>
       <c r="D26">
-        <v>379</v>
+        <v>400</v>
       </c>
       <c r="E26">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="F26">
-        <v>54</v>
+        <v>41</v>
       </c>
       <c r="G26">
         <v>2962576</v>
       </c>
       <c r="H26">
-        <v>210120</v>
+        <v>677475</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -56927,19 +56927,19 @@
         <v>1.5</v>
       </c>
       <c r="D27">
-        <v>356</v>
+        <v>377</v>
       </c>
       <c r="E27">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="F27">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G27">
         <v>2962576</v>
       </c>
       <c r="H27">
-        <v>210120</v>
+        <v>677475</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -56953,10 +56953,10 @@
         <v>2</v>
       </c>
       <c r="D28">
-        <v>306</v>
+        <v>332</v>
       </c>
       <c r="E28">
-        <v>181</v>
+        <v>155</v>
       </c>
       <c r="F28">
         <v>0</v>
@@ -56965,7 +56965,7 @@
         <v>2962576</v>
       </c>
       <c r="H28">
-        <v>210120</v>
+        <v>658603</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -56979,19 +56979,19 @@
         <v>1.25</v>
       </c>
       <c r="D29">
-        <v>379</v>
+        <v>387</v>
       </c>
       <c r="E29">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="F29">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="G29">
         <v>3068757</v>
       </c>
       <c r="H29">
-        <v>210120</v>
+        <v>619354</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -57005,19 +57005,19 @@
         <v>1.5</v>
       </c>
       <c r="D30">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="E30">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F30">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G30">
         <v>3068757</v>
       </c>
       <c r="H30">
-        <v>210120</v>
+        <v>619354</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -57031,10 +57031,10 @@
         <v>2</v>
       </c>
       <c r="D31">
-        <v>306</v>
+        <v>314</v>
       </c>
       <c r="E31">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="F31">
         <v>0</v>
@@ -57043,7 +57043,7 @@
         <v>3068757</v>
       </c>
       <c r="H31">
-        <v>210120</v>
+        <v>585839</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fiks 4 feil i analysescript, oppdater sensitivitetsdata og rapport
- ABC fallback: trigger også for TOTAL_NETWR <= 0, ikkje berre NaN (D-07)
- Sensitivitetsanalyse: reberekn kandidatsett per scenario i staden for
  å låse til base-case (OVERFØR_HVFS ∩ FOR_MANGE_ORDRER)
- K-means: legg til 7. farge for K=7 (hindrar IndexError)
- ABC/XYZ-oppsummering: fillna(0) etter reindex (hindrar int(NaN)-krasj)
- Rapport § 7.6 og § 9.1: legg til B_HVFS sensitivitetsrange (176–764 T)
- Word-dokument regenerert

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/006 Analyse/LOG650_Resultater.xlsx
+++ b/006 Analyse/LOG650_Resultater.xlsx
@@ -56367,7 +56367,7 @@
         <v>1602464</v>
       </c>
       <c r="H5">
-        <v>284941</v>
+        <v>286442</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -56601,7 +56601,7 @@
         <v>2221932</v>
       </c>
       <c r="H14">
-        <v>508107</v>
+        <v>515239</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -56627,7 +56627,7 @@
         <v>2221932</v>
       </c>
       <c r="H15">
-        <v>508107</v>
+        <v>513427</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -56679,7 +56679,7 @@
         <v>2333433</v>
       </c>
       <c r="H17">
-        <v>451519</v>
+        <v>454586</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -56757,7 +56757,7 @@
         <v>2481499</v>
       </c>
       <c r="H20">
-        <v>405479</v>
+        <v>406628</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -56835,7 +56835,7 @@
         <v>2898617</v>
       </c>
       <c r="H23">
-        <v>747776</v>
+        <v>763903</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -56861,7 +56861,7 @@
         <v>2898617</v>
       </c>
       <c r="H24">
-        <v>747776</v>
+        <v>761939</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -56913,7 +56913,7 @@
         <v>2962576</v>
       </c>
       <c r="H26">
-        <v>677475</v>
+        <v>686985</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -56939,7 +56939,7 @@
         <v>2962576</v>
       </c>
       <c r="H27">
-        <v>677475</v>
+        <v>684569</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -56991,7 +56991,7 @@
         <v>3068757</v>
       </c>
       <c r="H29">
-        <v>619354</v>
+        <v>624608</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -57017,7 +57017,7 @@
         <v>3068757</v>
       </c>
       <c r="H30">
-        <v>619354</v>
+        <v>620373</v>
       </c>
     </row>
     <row r="31" spans="1:8">

</xml_diff>